<commit_message>
Latest updates to the codes
Updated the most recent versions of the codes.
</commit_message>
<xml_diff>
--- a/Si_diamond_v2/silicon_formation_energies.xlsx
+++ b/Si_diamond_v2/silicon_formation_energies.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jdv/Desktop/Tulane/Tulane-Research/Projects/Defects_SCAN/fcc_metals_vac_formation_energy/updated_ingredients_March7/Silicon/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jdv/Documents/GitHub/dft_ingredients_analysis/Si_diamond_v2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCB9D4FF-040A-C740-AEEB-1FD047CD3227}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD145E8F-F131-B448-8FFE-E38544BFC2FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="20480" windowHeight="11520" xr2:uid="{E1340DD4-CBC3-4B48-B4E9-09C1BF3576B7}"/>
+    <workbookView xWindow="8720" yWindow="1240" windowWidth="20480" windowHeight="11520" xr2:uid="{E1340DD4-CBC3-4B48-B4E9-09C1BF3576B7}"/>
   </bookViews>
   <sheets>
     <sheet name="table_plot" sheetId="1" r:id="rId1"/>
@@ -492,13 +492,13 @@
         <v>0</v>
       </c>
       <c r="B2" s="2">
-        <v>3.42</v>
+        <v>3.38</v>
       </c>
       <c r="C2" s="2">
-        <v>3.39</v>
+        <v>3.36</v>
       </c>
       <c r="D2" s="2">
-        <v>3.33</v>
+        <v>3.49</v>
       </c>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>

</xml_diff>